<commit_message>
Update Address.line mappings with extensions for streetName and houseNumber b7fd67a02fcacff83b85373f20ede8b918f6c89c
</commit_message>
<xml_diff>
--- a/fsh/ig/CdaToAddressConceptMap.xlsx
+++ b/fsh/ig/CdaToAddressConceptMap.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="55">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-13T09:05:14+00:00</t>
+    <t>2026-04-13T09:40:13+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -159,7 +159,19 @@
     <t>AD.item.streetName</t>
   </si>
   <si>
+    <t>Address.line.extension.iso21090-ADXP-streetName</t>
+  </si>
+  <si>
+    <t>Address.line.extension[http://hl7.org/fhir/StructureDefinition/iso21090-ADXP-streetName]</t>
+  </si>
+  <si>
     <t>AD.item.houseNumber</t>
+  </si>
+  <si>
+    <t>Address.line.extension.iso21090-ADXP-houseNumber</t>
+  </si>
+  <si>
+    <t>Address.line.extension[http://hl7.org/fhir/StructureDefinition/iso21090-ADXP-houseNumber]</t>
   </si>
   <si>
     <t>AD.useablePeriod</t>
@@ -568,47 +580,47 @@
         <v>47</v>
       </c>
       <c r="C9" t="s" s="2">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E9" t="s" s="2">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="E10" t="s" s="2">
-        <v>46</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C11" t="s" s="2">
         <v>39</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E11" t="s" s="2">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update comments and target references in CdaToAddressConceptMap e260a49c9570f437c53575fae9e7b0d4d041a379
</commit_message>
<xml_diff>
--- a/fsh/ig/CdaToAddressConceptMap.xlsx
+++ b/fsh/ig/CdaToAddressConceptMap.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-13T09:58:36+00:00</t>
+    <t>2026-04-13T12:10:29+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -159,19 +159,19 @@
     <t>AD.item.streetName</t>
   </si>
   <si>
-    <t>Address.line.extension.iso21090-ADXP-streetName</t>
-  </si>
-  <si>
-    <t>Address.line.extension[http://hl7.org/fhir/StructureDefinition/iso21090-ADXP-streetName]</t>
+    <t>Address.line.extension[iso21090-ADXP-streetName].valueString</t>
+  </si>
+  <si>
+    <t>Address.line.extension[http://hl7.org/fhir/StructureDefinition/iso21090-ADXP-streetName].valueString</t>
   </si>
   <si>
     <t>AD.item.houseNumber</t>
   </si>
   <si>
-    <t>Address.line.extension.iso21090-ADXP-houseNumber</t>
-  </si>
-  <si>
-    <t>Address.line.extension[http://hl7.org/fhir/StructureDefinition/iso21090-ADXP-houseNumber]</t>
+    <t>Address.line.extension[iso21090-ADXP-houseNumber].valueString</t>
+  </si>
+  <si>
+    <t>Address.line.extension[http://hl7.org/fhir/StructureDefinition/iso21090-ADXP-houseNumber].valueString</t>
   </si>
   <si>
     <t>AD.useablePeriod</t>

</xml_diff>